<commit_message>
Added Merton Model for Credit Risk. Also updated dashboard with both methods.
</commit_message>
<xml_diff>
--- a/Merton Model.xlsx
+++ b/Merton Model.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/luism/Desktop/8-ITESO/Módelos de Crédito/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E30FCABA-0A0C-8E49-8581-432515679349}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE7ECD4-BCAB-E44B-B392-61B1A41CE33A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{32392DCD-070E-EC43-B159-7EFFE87224E1}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -127,13 +127,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -616,7 +619,7 @@
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="6">
         <v>100</v>
       </c>
     </row>
@@ -624,7 +627,7 @@
       <c r="B3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2">
+      <c r="C3" s="7">
         <v>60</v>
       </c>
     </row>
@@ -632,7 +635,7 @@
       <c r="B4" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="3">
+      <c r="C4" s="8">
         <v>0.03</v>
       </c>
     </row>
@@ -640,7 +643,7 @@
       <c r="B5" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="8">
         <v>0.2</v>
       </c>
     </row>

</xml_diff>